<commit_message>
The platform's mail server carries the platform's own mail only; every tenant has its own (patch 0027)
Sharing the platform row with tenants is gone: no "Sharing with tenants" in the back-office, no "Use the Platform's Mail Server" under Settings -> Email Server, and the campaign SMTP engine only ever opens the tenant's own server. The platform server sends alerts and back-office password links, and stands in for a tenant that has no working server of its own. Patch 0027 drops the sharing columns; a tenant row that sent through the platform server is removed with its campaign sender.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CEP_Tenant_Onboarding_and_Sending_Setup.xlsx
+++ b/docs/CEP_Tenant_Onboarding_and_Sending_Setup.xlsx
@@ -846,17 +846,17 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Back-office → Email server</t>
+          <t>Back-office → Mail server</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>An SMTP server the platform uses for its own notifications, shareable with workspaces as a campaign sender.</t>
+          <t>An SMTP server for the platform's own mail only: alerts, password links, and the fallback for a workspace that has not entered its own server yet.</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>Optional: a workspace can bring its own engine instead (sheet 3).</t>
+          <t>Never a workspace's sending engine: every workspace enters its own mail server or sending engine (sheet 3).</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
@@ -1940,7 +1940,7 @@
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>Also usable as the platform's shared server (back-office).</t>
+          <t>Each workspace has its own; the platform's server is not offered.</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">

</xml_diff>